<commit_message>
Classificaiton task for project validation
</commit_message>
<xml_diff>
--- a/SFT/LoRa/lora_sft_model_comparison.xlsx
+++ b/SFT/LoRa/lora_sft_model_comparison.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WINDOWS 11\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\SEM-7\Capstone\SFT\LoRa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1A3D318-3DD5-4F56-B58B-C99213D4A193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{552B0BAA-2CDF-4DDE-9635-47AB26C281AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Red Team Comparison" sheetId="1" r:id="rId1"/>
-    <sheet name="Blue Team Comparison" sheetId="2" r:id="rId2"/>
-    <sheet name="Red Loss Curve" sheetId="3" r:id="rId3"/>
+    <sheet name="Red Loss Curve" sheetId="3" r:id="rId2"/>
+    <sheet name="Blue Team Comparison" sheetId="2" r:id="rId3"/>
     <sheet name="Blue Loss Curve" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
@@ -295,17 +295,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -345,9 +336,17 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1997,427 +1996,424 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="17"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="3" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="3">
         <v>7608</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="3">
         <v>7608</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="3">
         <v>7608</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="6" t="b">
+      <c r="B7" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="C7" s="6" t="b">
+      <c r="C7" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="D7" s="6" t="b">
+      <c r="D7" s="3" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="3">
         <v>3</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="3">
         <v>3</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="3">
         <v>1</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="3">
         <v>1</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="3">
         <v>16</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="3">
         <v>16</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="3">
         <v>69</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="3">
         <v>69</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="3">
         <v>28</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="3">
         <v>36</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="3">
         <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="6">
+      <c r="B13" s="3">
         <v>32</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="3">
         <v>32</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="3">
         <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="3">
         <v>64</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="3">
         <v>64</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="3">
         <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15" s="4">
         <v>0.05</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="4">
         <v>0.05</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="4">
         <v>0.05</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="5">
         <v>80740352</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="5">
         <v>87293952</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="5">
         <v>83886080</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="5">
         <v>4972287488</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="5">
         <v>5279101952</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="5">
         <v>4712566784</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="6">
         <f>B16/B17</f>
         <v>1.6238069941622812E-2</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="6">
         <f>C16/C17</f>
         <v>1.6535757936428655E-2</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="6">
         <f>D16/D17</f>
         <v>1.7800507418761283E-2</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="7">
         <v>2.034192</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="7">
         <v>2.1346560000000001</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="7">
         <v>1.832441</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="7">
         <v>1.491079</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="7">
         <v>1.4956199999999999</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="7">
         <v>1.3840859999999999</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="7">
         <v>1.2194929999999999</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="7">
         <v>1.2526109999999999</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="7">
         <v>1.0746789999999999</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="7">
         <v>1.0507470000000001</v>
       </c>
-      <c r="C22" s="10">
+      <c r="C22" s="7">
         <v>1.121248</v>
       </c>
-      <c r="D22" s="10">
+      <c r="D22" s="7">
         <v>0.93673499999999998</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="7">
         <v>0.90023500000000001</v>
       </c>
-      <c r="C23" s="10">
+      <c r="C23" s="7">
         <v>0.97016199999999997</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="7">
         <v>0.78131499999999998</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="7">
         <v>0.77592499999999998</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C24" s="7">
         <v>0.87440700000000005</v>
       </c>
-      <c r="D24" s="10">
+      <c r="D24" s="7">
         <v>0.62920600000000004</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="10">
+      <c r="B25" s="7">
         <v>1.1857</v>
       </c>
-      <c r="C25" s="10">
+      <c r="C25" s="7">
         <v>1.2529999999999999</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="8">
         <v>1.0478000000000001</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="12">
+      <c r="B26" s="9">
         <f>(B19-B25)/B19</f>
         <v>0.41711500192705508</v>
       </c>
-      <c r="C26" s="12">
+      <c r="C26" s="9">
         <f>(C19-C25)/C19</f>
         <v>0.41302017748995629</v>
       </c>
-      <c r="D26" s="12">
+      <c r="D26" s="9">
         <f>(D19-D25)/D19</f>
         <v>0.42819441389927421</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="10">
         <v>280.01</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C27" s="4">
         <v>380.55</v>
       </c>
-      <c r="D27" s="7">
+      <c r="D27" s="4">
         <v>344.98</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="10">
         <v>4.67</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="4">
         <v>6.34</v>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="4">
         <v>5.75</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="4">
         <f>B27/B11</f>
         <v>4.0581159420289854</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="4">
         <f>C27/C11</f>
         <v>5.5152173913043478</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="4">
         <f>D27/D11</f>
         <v>4.9997101449275361</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="4">
         <f>B27/B8</f>
         <v>93.336666666666659</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="4">
         <f>C27/C8</f>
         <v>126.85000000000001</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="4">
         <f>D27/D8</f>
         <v>114.99333333333334</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2430,459 +2426,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D33"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="4" width="40" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="3" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="6">
-        <v>7608</v>
-      </c>
-      <c r="C6" s="6">
-        <v>7608</v>
-      </c>
-      <c r="D6" s="6">
-        <v>7608</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="6">
-        <v>3</v>
-      </c>
-      <c r="C8" s="6">
-        <v>3</v>
-      </c>
-      <c r="D8" s="6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="6">
-        <v>1</v>
-      </c>
-      <c r="C9" s="6">
-        <v>1</v>
-      </c>
-      <c r="D9" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="6">
-        <v>16</v>
-      </c>
-      <c r="C10" s="6">
-        <v>16</v>
-      </c>
-      <c r="D10" s="6">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="6">
-        <v>72</v>
-      </c>
-      <c r="C11" s="6">
-        <v>72</v>
-      </c>
-      <c r="D11" s="6">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="6">
-        <v>28</v>
-      </c>
-      <c r="C12" s="6">
-        <v>36</v>
-      </c>
-      <c r="D12" s="6">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="6">
-        <v>32</v>
-      </c>
-      <c r="C13" s="6">
-        <v>32</v>
-      </c>
-      <c r="D13" s="6">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="6">
-        <v>64</v>
-      </c>
-      <c r="C14" s="6">
-        <v>64</v>
-      </c>
-      <c r="D14" s="6">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="7">
-        <v>0.05</v>
-      </c>
-      <c r="C15" s="7">
-        <v>0.05</v>
-      </c>
-      <c r="D15" s="7">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="8">
-        <v>80740352</v>
-      </c>
-      <c r="C16" s="8">
-        <v>87293952</v>
-      </c>
-      <c r="D16" s="8">
-        <v>83886080</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="8">
-        <v>4972287488</v>
-      </c>
-      <c r="C17" s="8">
-        <v>5279101952</v>
-      </c>
-      <c r="D17" s="8">
-        <v>4712566784</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="9">
-        <f>B16/B17</f>
-        <v>1.6238069941622812E-2</v>
-      </c>
-      <c r="C18" s="9">
-        <f>C16/C17</f>
-        <v>1.6535757936428655E-2</v>
-      </c>
-      <c r="D18" s="9">
-        <f>D16/D17</f>
-        <v>1.7800507418761283E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="10">
-        <v>2.0398230000000002</v>
-      </c>
-      <c r="C19" s="10">
-        <v>2.1931289999999999</v>
-      </c>
-      <c r="D19" s="10">
-        <v>1.8987019999999999</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" s="10">
-        <v>1.5163709999999999</v>
-      </c>
-      <c r="C20" s="10">
-        <v>1.5362309999999999</v>
-      </c>
-      <c r="D20" s="10">
-        <v>1.3997839999999999</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="10">
-        <v>1.1962520000000001</v>
-      </c>
-      <c r="C21" s="10">
-        <v>1.2443869999999999</v>
-      </c>
-      <c r="D21" s="10">
-        <v>1.10859</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="10">
-        <v>1.0577460000000001</v>
-      </c>
-      <c r="C22" s="10">
-        <v>1.133405</v>
-      </c>
-      <c r="D22" s="10">
-        <v>0.953376</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B23" s="10">
-        <v>1.0418510000000001</v>
-      </c>
-      <c r="C23" s="10">
-        <v>1.111192</v>
-      </c>
-      <c r="D23" s="10">
-        <v>0.84875800000000001</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24" s="10">
-        <v>0.78368400000000005</v>
-      </c>
-      <c r="C24" s="10">
-        <v>0.87799499999999997</v>
-      </c>
-      <c r="D24" s="10">
-        <v>0.60974200000000001</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B25" s="10">
-        <v>0.76998699999999998</v>
-      </c>
-      <c r="C25" s="10">
-        <v>0.87429199999999996</v>
-      </c>
-      <c r="D25" s="10">
-        <v>0.642181</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="10">
-        <v>1.1872</v>
-      </c>
-      <c r="C26" s="10">
-        <v>1.2688999999999999</v>
-      </c>
-      <c r="D26" s="11">
-        <v>1.0552999999999999</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" s="12">
-        <f>(B19-B26)/B19</f>
-        <v>0.41798871764854112</v>
-      </c>
-      <c r="C27" s="12">
-        <f>(C19-C26)/C19</f>
-        <v>0.42142026301234448</v>
-      </c>
-      <c r="D27" s="12">
-        <f>(D19-D26)/D19</f>
-        <v>0.44419924769658431</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28" s="13">
-        <v>288.89</v>
-      </c>
-      <c r="C28" s="7">
-        <v>358.37</v>
-      </c>
-      <c r="D28" s="7">
-        <v>354.32</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B29" s="13">
-        <v>4.8099999999999996</v>
-      </c>
-      <c r="C29" s="7">
-        <v>5.97</v>
-      </c>
-      <c r="D29" s="7">
-        <v>5.91</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B30" s="7">
-        <f>B28/B11</f>
-        <v>4.0123611111111108</v>
-      </c>
-      <c r="C30" s="7">
-        <f>C28/C11</f>
-        <v>4.9773611111111116</v>
-      </c>
-      <c r="D30" s="7">
-        <f>D28/D11</f>
-        <v>4.9211111111111112</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B31" s="7">
-        <f>B28/B8</f>
-        <v>96.296666666666667</v>
-      </c>
-      <c r="C31" s="7">
-        <f>C28/C8</f>
-        <v>119.45666666666666</v>
-      </c>
-      <c r="D31" s="7">
-        <f>D28/D8</f>
-        <v>118.10666666666667</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A33:D33"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2894,108 +2437,108 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
     </row>
     <row r="3" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="14">
+      <c r="A4" s="11">
         <v>10</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="12">
         <v>2.034192</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="12">
         <v>2.1346560000000001</v>
       </c>
-      <c r="D4" s="15">
+      <c r="D4" s="12">
         <v>1.832441</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="14">
+      <c r="A5" s="11">
         <v>20</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="12">
         <v>1.491079</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="12">
         <v>1.4956199999999999</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="12">
         <v>1.3840859999999999</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="14">
+      <c r="A6" s="11">
         <v>30</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="12">
         <v>1.2194929999999999</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="12">
         <v>1.2526109999999999</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="12">
         <v>1.0746789999999999</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="14">
+      <c r="A7" s="11">
         <v>40</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="12">
         <v>1.0507470000000001</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="12">
         <v>1.121248</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="12">
         <v>0.93673499999999998</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="14">
+      <c r="A8" s="11">
         <v>50</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="12">
         <v>0.90023500000000001</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="12">
         <v>0.97016199999999997</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="12">
         <v>0.78131499999999998</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="14">
+      <c r="A9" s="11">
         <v>60</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="12">
         <v>0.77592499999999998</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="12">
         <v>0.87440700000000005</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="12">
         <v>0.62920600000000004</v>
       </c>
     </row>
@@ -3006,6 +2549,459 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="4" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+    </row>
+    <row r="3" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="3">
+        <v>7608</v>
+      </c>
+      <c r="C6" s="3">
+        <v>7608</v>
+      </c>
+      <c r="D6" s="3">
+        <v>7608</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3">
+        <v>3</v>
+      </c>
+      <c r="C8" s="3">
+        <v>3</v>
+      </c>
+      <c r="D8" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="3">
+        <v>1</v>
+      </c>
+      <c r="C9" s="3">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="3">
+        <v>16</v>
+      </c>
+      <c r="C10" s="3">
+        <v>16</v>
+      </c>
+      <c r="D10" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="3">
+        <v>72</v>
+      </c>
+      <c r="C11" s="3">
+        <v>72</v>
+      </c>
+      <c r="D11" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="3">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3">
+        <v>36</v>
+      </c>
+      <c r="D12" s="3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="3">
+        <v>32</v>
+      </c>
+      <c r="C13" s="3">
+        <v>32</v>
+      </c>
+      <c r="D13" s="3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="3">
+        <v>64</v>
+      </c>
+      <c r="C14" s="3">
+        <v>64</v>
+      </c>
+      <c r="D14" s="3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="5">
+        <v>80740352</v>
+      </c>
+      <c r="C16" s="5">
+        <v>87293952</v>
+      </c>
+      <c r="D16" s="5">
+        <v>83886080</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="5">
+        <v>4972287488</v>
+      </c>
+      <c r="C17" s="5">
+        <v>5279101952</v>
+      </c>
+      <c r="D17" s="5">
+        <v>4712566784</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="6">
+        <f>B16/B17</f>
+        <v>1.6238069941622812E-2</v>
+      </c>
+      <c r="C18" s="6">
+        <f>C16/C17</f>
+        <v>1.6535757936428655E-2</v>
+      </c>
+      <c r="D18" s="6">
+        <f>D16/D17</f>
+        <v>1.7800507418761283E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="7">
+        <v>2.0398230000000002</v>
+      </c>
+      <c r="C19" s="7">
+        <v>2.1931289999999999</v>
+      </c>
+      <c r="D19" s="7">
+        <v>1.8987019999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="7">
+        <v>1.5163709999999999</v>
+      </c>
+      <c r="C20" s="7">
+        <v>1.5362309999999999</v>
+      </c>
+      <c r="D20" s="7">
+        <v>1.3997839999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="7">
+        <v>1.1962520000000001</v>
+      </c>
+      <c r="C21" s="7">
+        <v>1.2443869999999999</v>
+      </c>
+      <c r="D21" s="7">
+        <v>1.10859</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="7">
+        <v>1.0577460000000001</v>
+      </c>
+      <c r="C22" s="7">
+        <v>1.133405</v>
+      </c>
+      <c r="D22" s="7">
+        <v>0.953376</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="7">
+        <v>1.0418510000000001</v>
+      </c>
+      <c r="C23" s="7">
+        <v>1.111192</v>
+      </c>
+      <c r="D23" s="7">
+        <v>0.84875800000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="7">
+        <v>0.78368400000000005</v>
+      </c>
+      <c r="C24" s="7">
+        <v>0.87799499999999997</v>
+      </c>
+      <c r="D24" s="7">
+        <v>0.60974200000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="7">
+        <v>0.76998699999999998</v>
+      </c>
+      <c r="C25" s="7">
+        <v>0.87429199999999996</v>
+      </c>
+      <c r="D25" s="7">
+        <v>0.642181</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="7">
+        <v>1.1872</v>
+      </c>
+      <c r="C26" s="7">
+        <v>1.2688999999999999</v>
+      </c>
+      <c r="D26" s="8">
+        <v>1.0552999999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" s="9">
+        <f>(B19-B26)/B19</f>
+        <v>0.41798871764854112</v>
+      </c>
+      <c r="C27" s="9">
+        <f>(C19-C26)/C19</f>
+        <v>0.42142026301234448</v>
+      </c>
+      <c r="D27" s="9">
+        <f>(D19-D26)/D19</f>
+        <v>0.44419924769658431</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" s="10">
+        <v>288.89</v>
+      </c>
+      <c r="C28" s="4">
+        <v>358.37</v>
+      </c>
+      <c r="D28" s="4">
+        <v>354.32</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="10">
+        <v>4.8099999999999996</v>
+      </c>
+      <c r="C29" s="4">
+        <v>5.97</v>
+      </c>
+      <c r="D29" s="4">
+        <v>5.91</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="4">
+        <f>B28/B11</f>
+        <v>4.0123611111111108</v>
+      </c>
+      <c r="C30" s="4">
+        <f>C28/C11</f>
+        <v>4.9773611111111116</v>
+      </c>
+      <c r="D30" s="4">
+        <f>D28/D11</f>
+        <v>4.9211111111111112</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="4">
+        <f>B28/B8</f>
+        <v>96.296666666666667</v>
+      </c>
+      <c r="C31" s="4">
+        <f>C28/C8</f>
+        <v>119.45666666666666</v>
+      </c>
+      <c r="D31" s="4">
+        <f>D28/D8</f>
+        <v>118.10666666666667</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A33:D33"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
@@ -3021,122 +3017,122 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
     </row>
     <row r="3" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="14">
+      <c r="A4" s="11">
         <v>10</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="12">
         <v>2.0398230000000002</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="12">
         <v>2.1931289999999999</v>
       </c>
-      <c r="D4" s="15">
+      <c r="D4" s="12">
         <v>1.8987019999999999</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="14">
+      <c r="A5" s="11">
         <v>20</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="12">
         <v>1.5163709999999999</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="12">
         <v>1.5362309999999999</v>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="12">
         <v>1.3997839999999999</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="14">
+      <c r="A6" s="11">
         <v>30</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="12">
         <v>1.1962520000000001</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="12">
         <v>1.2443869999999999</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="12">
         <v>1.10859</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="14">
+      <c r="A7" s="11">
         <v>40</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="12">
         <v>1.0577460000000001</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="12">
         <v>1.133405</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="12">
         <v>0.953376</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="14">
+      <c r="A8" s="11">
         <v>50</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="12">
         <v>1.0418510000000001</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="12">
         <v>1.111192</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="12">
         <v>0.84875800000000001</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="14">
+      <c r="A9" s="11">
         <v>60</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="12">
         <v>0.78368400000000005</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="12">
         <v>0.87799499999999997</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="12">
         <v>0.60974200000000001</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="14">
+      <c r="A10" s="11">
         <v>70</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="12">
         <v>0.76998699999999998</v>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="12">
         <v>0.87429199999999996</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="12">
         <v>0.642181</v>
       </c>
     </row>

</xml_diff>